<commit_message>
Protect downloadable Excel workbooks
</commit_message>
<xml_diff>
--- a/public/work-samples/apple-financial-model.xlsx
+++ b/public/work-samples/apple-financial-model.xlsx
@@ -18774,6 +18774,7 @@
       <c r="W52" s="162"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="12">
     <mergeCell ref="B2:O2"/>
     <mergeCell ref="K10:O10"/>
@@ -19856,6 +19857,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -20508,6 +20510,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="3">
     <mergeCell ref="G30:K30"/>
     <mergeCell ref="B23:E23"/>
@@ -21367,6 +21370,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="5">
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="O8:Q8"/>
@@ -32167,6 +32171,7 @@
       <c r="G486" s="3"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="3">
     <mergeCell ref="B6:L6"/>
     <mergeCell ref="I8:L8"/>
@@ -33006,6 +33011,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="6">
     <mergeCell ref="B67:K67"/>
     <mergeCell ref="B26:K26"/>
@@ -33038,6 +33044,7 @@
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
   </cols>
   <sheetData/>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
@@ -47341,6 +47348,7 @@
       <c r="B947"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -47358,6 +47366,7 @@
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
   </cols>
   <sheetData/>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
@@ -55170,6 +55179,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="8">
     <mergeCell ref="B114:R114"/>
     <mergeCell ref="B63:R63"/>
@@ -55939,6 +55949,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="3">
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="G6:J6"/>
@@ -57928,6 +57939,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="2">
     <mergeCell ref="B6:M6"/>
     <mergeCell ref="N6:O6"/>
@@ -60234,6 +60246,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="2">
     <mergeCell ref="B6:L6"/>
     <mergeCell ref="B24:L24"/>
@@ -60255,6 +60268,7 @@
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
   </cols>
   <sheetData/>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
@@ -60842,6 +60856,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="1">
     <mergeCell ref="B6:J6"/>
   </mergeCells>
@@ -64921,6 +64936,7 @@
       <c r="AA70" s="3"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="7">
     <mergeCell ref="U8:W8"/>
     <mergeCell ref="Y8:AA8"/>

</xml_diff>

<commit_message>
Add worksheet editing passwords
</commit_message>
<xml_diff>
--- a/public/work-samples/apple-financial-model.xlsx
+++ b/public/work-samples/apple-financial-model.xlsx
@@ -18774,7 +18774,7 @@
       <c r="W52" s="162"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="12">
     <mergeCell ref="B2:O2"/>
     <mergeCell ref="K10:O10"/>
@@ -19857,7 +19857,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -20510,7 +20510,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="3">
     <mergeCell ref="G30:K30"/>
     <mergeCell ref="B23:E23"/>
@@ -21370,7 +21370,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="5">
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="O8:Q8"/>
@@ -32171,7 +32171,7 @@
       <c r="G486" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="3">
     <mergeCell ref="B6:L6"/>
     <mergeCell ref="I8:L8"/>
@@ -33011,7 +33011,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="6">
     <mergeCell ref="B67:K67"/>
     <mergeCell ref="B26:K26"/>
@@ -33044,7 +33044,7 @@
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
   </cols>
   <sheetData/>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
@@ -47348,7 +47348,7 @@
       <c r="B947"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -47366,7 +47366,7 @@
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
   </cols>
   <sheetData/>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
@@ -55179,7 +55179,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="8">
     <mergeCell ref="B114:R114"/>
     <mergeCell ref="B63:R63"/>
@@ -55949,7 +55949,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="3">
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="G6:J6"/>
@@ -57939,7 +57939,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="2">
     <mergeCell ref="B6:M6"/>
     <mergeCell ref="N6:O6"/>
@@ -60246,7 +60246,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="2">
     <mergeCell ref="B6:L6"/>
     <mergeCell ref="B24:L24"/>
@@ -60268,7 +60268,7 @@
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
   </cols>
   <sheetData/>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
@@ -60856,7 +60856,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="1">
     <mergeCell ref="B6:J6"/>
   </mergeCells>
@@ -64936,7 +64936,7 @@
       <c r="AA70" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <sheetProtection password="CC0B" sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
   <mergeCells count="7">
     <mergeCell ref="U8:W8"/>
     <mergeCell ref="Y8:AA8"/>

</xml_diff>